<commit_message>
Added all subject modals & json files
</commit_message>
<xml_diff>
--- a/CLASS/SS1/Chemistry/results.xlsx
+++ b/CLASS/SS1/Chemistry/results.xlsx
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aliyu Ahmad</t>
+          <t>Salisu Nana Asmau</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>std153</t>
+          <t>std143</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SS1B</t>
+          <t>SS1_SILVER</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,11 +486,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
         <v>50</v>
@@ -502,7 +502,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2025-12-03 11:03</t>
+          <t>2025-12-06 23:26</t>
         </is>
       </c>
     </row>

</xml_diff>